<commit_message>
docs(sprint5): report, progress, conformance and final evidence
</commit_message>
<xml_diff>
--- a/acceptance-evidence/dual-system-v1/tests/sprint5/files/big.xlsx
+++ b/acceptance-evidence/dual-system-v1/tests/sprint5/files/big.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>2026-09-12T12:48:16.762Z</t>
+          <t>2026-09-12T13:41:44.825Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sprint5): record final build sha e639707 and refreshed evidence
</commit_message>
<xml_diff>
--- a/acceptance-evidence/dual-system-v1/tests/sprint5/files/big.xlsx
+++ b/acceptance-evidence/dual-system-v1/tests/sprint5/files/big.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>2026-09-12T13:41:44.825Z</t>
+          <t>2026-09-12T13:49:38.887Z</t>
         </is>
       </c>
     </row>

</xml_diff>